<commit_message>
Replace placeholder exported documents
</commit_message>
<xml_diff>
--- a/assets/docs/financial_model.xlsx
+++ b/assets/docs/financial_model.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COGS_Opex" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profitability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_View" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +32,37 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="001F2A36"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2A36"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E2A3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF4E7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +70,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D7D0C5"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D7D0C5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7D0C5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D7D0C5"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,161 +479,704 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Audience</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Conversion Rate</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Orders</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Average Order Value</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Audience Year 1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Combined social and owned audience</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Audience Year 2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Scaled through content and launches</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Audience Year 3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Brand authority and partnerships</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Collections Year 1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Quarterly launch cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Collections Year 2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Bi-monthly cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Collections Year 3</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Monthly launch cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ASP Year 1</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Premium entry assortment</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ASP Year 2</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Expanded premium mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ASP Year 3</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Private label and richer assortment</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Gross Margin Target Low</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Conservative blended margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Gross Margin Target High</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Private label upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Membership Price</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Passport Club monthly price</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Collections launched</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Total units sold</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Average selling price</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Product revenue</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>650000</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>6912000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Membership revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>96000</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>480000</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1440000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Partnership + affiliate</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>80000</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>320000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>826000</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>9352000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Gross Profit</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Operating Cost</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Net Profit</t>
+      <c r="B2" s="6" t="n">
+        <v>280000</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>1120000</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>2688000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Travel and sourcing</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Marketing and growth</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>82600</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>432000</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1028720</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>General operations</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Total operating costs</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>367600</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>1147000</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>2398720</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Year 3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Month1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>65</v>
-      </c>
-      <c r="F2" t="n">
-        <v>6500</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2800</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3700</v>
-      </c>
-      <c r="I2" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1700</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>826000</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>9352000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Month2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="D3" t="n">
-        <v>180</v>
-      </c>
-      <c r="E3" t="n">
-        <v>65</v>
-      </c>
-      <c r="F3" t="n">
-        <v>11700</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>6700</v>
-      </c>
-      <c r="I3" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J3" t="n">
-        <v>4200</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>COGS</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>280000</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>1120000</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>2688000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Month3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="D4" t="n">
-        <v>300</v>
-      </c>
-      <c r="E4" t="n">
-        <v>65</v>
-      </c>
-      <c r="F4" t="n">
-        <v>19500</v>
-      </c>
-      <c r="G4" t="n">
-        <v>8400</v>
-      </c>
-      <c r="H4" t="n">
-        <v>11100</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>8100</v>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Gross profit</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>546000</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>2480000</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>6664000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Total operating costs</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>367600</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>1147000</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>2398720</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Indicative operating profit</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>178400</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>1333000</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>4265280</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year 3 Revenue</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Commentary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Base case</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>9352000</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Current planning case</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Upside case</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Faster repeat purchase and earlier private label expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Downside case</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Slower audience growth and lower sell-through</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>